<commit_message>
DataSchema nonlinkage mortality updated V2
</commit_message>
<xml_diff>
--- a/mortality/dataschema_ProPASS_mortality.xlsx
+++ b/mortality/dataschema_ProPASS_mortality.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\DataSchemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{41B3C7EB-4832-4A36-9BDE-3265CEB528EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E89D243B-190D-47B5-9138-8EDA9779A223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DB9EE49B-F8BF-4815-B441-B0BA94DBFC22}"/>
+    <workbookView xWindow="-28920" yWindow="1620" windowWidth="29040" windowHeight="15720" xr2:uid="{DB9EE49B-F8BF-4815-B441-B0BA94DBFC22}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="65">
   <si>
     <t>index</t>
   </si>
@@ -78,9 +78,6 @@
     <t>source</t>
   </si>
   <si>
-    <t>wording</t>
-  </si>
-  <si>
     <t>instructions</t>
   </si>
   <si>
@@ -186,12 +183,6 @@
     <t>Death date - Year</t>
   </si>
   <si>
-    <t>questionnaire; mortality registry; familly survey</t>
-  </si>
-  <si>
-    <t>propass_mortality_1_0</t>
-  </si>
-  <si>
     <t>adm_collect_year</t>
   </si>
   <si>
@@ -213,13 +204,37 @@
     <t>Study country</t>
   </si>
   <si>
-    <t>Time of data collect - Year component, to inform censoring</t>
-  </si>
-  <si>
-    <t>Time of data collect - Month component, to inform censoring</t>
-  </si>
-  <si>
     <t>Note the source of the information about data collection time, e.g., if it comes from the study or is based on the collection event.</t>
+  </si>
+  <si>
+    <t>propass_nonlinkage_mortality_1_0</t>
+  </si>
+  <si>
+    <t>cohort documentation</t>
+  </si>
+  <si>
+    <t>yyyy</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>dd</t>
+  </si>
+  <si>
+    <t>adm_months_followup</t>
+  </si>
+  <si>
+    <t>Months of follow-up</t>
+  </si>
+  <si>
+    <t>Number of months of participant follow-up from baseline</t>
+  </si>
+  <si>
+    <t>months</t>
+  </si>
+  <si>
+    <t>If this is calculated from difference between two dates, round to nearest whole month.</t>
   </si>
 </sst>
 </file>
@@ -269,9 +284,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -606,19 +627,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F8E0180-A72F-4AF4-960B-1515820225EB}">
-  <dimension ref="A1:O11"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:N12"/>
+  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="55.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" customWidth="1"/>
+    <col min="4" max="4" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="43.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -661,260 +684,269 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" t="s">
+      <c r="J2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" t="s">
+      <c r="M2" t="s">
         <v>20</v>
       </c>
-      <c r="N2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
         <v>22</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>23</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" t="s">
         <v>24</v>
       </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="M3" t="s">
         <v>25</v>
       </c>
-      <c r="N3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
         <v>27</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>28</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" t="s">
         <v>29</v>
       </c>
-      <c r="G4" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="M4" t="s">
         <v>30</v>
       </c>
-      <c r="N4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" t="s">
         <v>49</v>
       </c>
-      <c r="D6" t="s">
-        <v>50</v>
-      </c>
-      <c r="E6" t="s">
-        <v>52</v>
-      </c>
       <c r="F6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" t="s">
+        <v>31</v>
+      </c>
+      <c r="I6" t="s">
         <v>57</v>
       </c>
-      <c r="G6" t="s">
+      <c r="J6" t="s">
         <v>32</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>33</v>
       </c>
-      <c r="K6" t="s">
-        <v>34</v>
-      </c>
-      <c r="N6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="M6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" t="s">
         <v>58</v>
       </c>
-      <c r="G7" t="s">
+      <c r="J7" t="s">
         <v>32</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>33</v>
       </c>
-      <c r="K7" t="s">
-        <v>34</v>
-      </c>
-      <c r="N7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="M7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>15</v>
+      <c r="B8" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" t="s">
-        <v>41</v>
-      </c>
-      <c r="G8" t="s">
-        <v>32</v>
-      </c>
-      <c r="J8" t="s">
-        <v>20</v>
+        <v>55</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="K8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E9" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="F9" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D10" t="s">
         <v>43</v>
@@ -926,48 +958,89 @@
         <v>46</v>
       </c>
       <c r="G10" t="s">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="I10" t="s">
+        <v>57</v>
       </c>
       <c r="J10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="L10" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" t="s">
+        <v>58</v>
+      </c>
+      <c r="J11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K11" t="s">
+        <v>33</v>
+      </c>
+      <c r="L11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" t="s">
         <v>44</v>
       </c>
-      <c r="E11" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" t="s">
-        <v>47</v>
-      </c>
-      <c r="G11" t="s">
-        <v>32</v>
-      </c>
-      <c r="J11" t="s">
-        <v>20</v>
-      </c>
-      <c r="K11" t="s">
-        <v>34</v>
-      </c>
-      <c r="L11" t="s">
-        <v>48</v>
+      <c r="F12" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" t="s">
+        <v>31</v>
+      </c>
+      <c r="I12" t="s">
+        <v>59</v>
+      </c>
+      <c r="J12" t="s">
+        <v>19</v>
+      </c>
+      <c r="K12" t="s">
+        <v>33</v>
+      </c>
+      <c r="L12" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -979,74 +1052,74 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D6186D5-BB84-4E3C-AAC4-F17A4EDF9A5A}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" t="b">
         <v>0</v>
       </c>
-      <c r="F2" t="s">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3">
+      <c r="F3" t="b">
         <v>0</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>